<commit_message>
refactor : modification du Tableau de synthese RUTH METAYER.xlsx
</commit_message>
<xml_diff>
--- a/public/Tableau de synthese RUTH METAYER.xlsx
+++ b/public/Tableau de synthese RUTH METAYER.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29819"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Shared/Examens, concours/BTS SIO/RS2024/Projet circulaire/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\SLAM\2\Ruthh-mt.github.io\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="95" documentId="8_{77A5C754-F932-1645-AFCC-C393A53F72B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65769130-E25E-4D56-BDD8-1DB442440423}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1668F915-C18E-488C-89B1-A0301A1DBD61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1380" yWindow="500" windowWidth="34460" windowHeight="21900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="52">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -249,7 +249,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -815,15 +815,39 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -855,30 +879,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1190,66 +1190,66 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AQ82"/>
-  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.42578125" customWidth="1"/>
-    <col min="44" max="16384" width="10.7109375" style="1"/>
+    <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="1" customWidth="1"/>
+    <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.44140625" customWidth="1"/>
+    <col min="44" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="29"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1">
-      <c r="A2" s="29" t="s">
+      <c r="H1" s="27"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-    </row>
-    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1">
-      <c r="A3" s="41" t="s">
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+    </row>
+    <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="47" t="s">
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="42"/>
-      <c r="H3" s="48"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="35"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1">
-      <c r="A4" s="44" t="s">
+    <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="46"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="33"/>
       <c r="F4" s="12" t="s">
         <v>6</v>
       </c>
@@ -1260,23 +1260,23 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1">
-      <c r="A5" s="38" t="s">
+    <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="39"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="40"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1">
-      <c r="A6" s="27" t="s">
+      <c r="B5" s="47"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="47"/>
+      <c r="G5" s="47"/>
+      <c r="H5" s="48"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="44" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1298,9 +1298,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1">
-      <c r="A7" s="28"/>
-      <c r="B7" s="37"/>
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="37"/>
+      <c r="B7" s="45"/>
       <c r="C7" s="19" t="s">
         <v>18</v>
       </c>
@@ -1355,17 +1355,17 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="18">
-      <c r="A8" s="30" t="s">
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A8" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="31"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="32"/>
+      <c r="B8" s="39"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1402,7 +1402,7 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>25</v>
       </c>
@@ -1455,7 +1455,7 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>29</v>
       </c>
@@ -1508,7 +1508,7 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>31</v>
       </c>
@@ -1561,7 +1561,7 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>33</v>
       </c>
@@ -1612,7 +1612,7 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>35</v>
       </c>
@@ -1663,7 +1663,7 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
         <v>37</v>
       </c>
@@ -1712,7 +1712,7 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>39</v>
       </c>
@@ -1722,7 +1722,9 @@
       <c r="C15" s="15"/>
       <c r="D15" s="15"/>
       <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
+      <c r="F15" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="G15" s="15"/>
       <c r="H15" s="16"/>
       <c r="I15"/>
@@ -1761,7 +1763,7 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>41</v>
       </c>
@@ -1810,7 +1812,7 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>43</v>
       </c>
@@ -1820,8 +1822,12 @@
       <c r="C17" s="15"/>
       <c r="D17" s="15"/>
       <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
+      <c r="F17" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="H17" s="16"/>
       <c r="I17"/>
       <c r="J17"/>
@@ -1859,7 +1865,7 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>45</v>
       </c>
@@ -1870,7 +1876,9 @@
       <c r="D18" s="15"/>
       <c r="E18" s="15"/>
       <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
+      <c r="G18" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="H18" s="16" t="s">
         <v>27</v>
       </c>
@@ -1910,7 +1918,7 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>47</v>
       </c>
@@ -1920,7 +1928,9 @@
       <c r="C19" s="15"/>
       <c r="D19" s="15"/>
       <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
+      <c r="F19" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="G19" s="15"/>
       <c r="H19" s="16"/>
       <c r="I19"/>
@@ -1959,17 +1969,17 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="18">
-      <c r="A20" s="33" t="s">
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A20" s="41" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="34"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="35"/>
+      <c r="B20" s="42"/>
+      <c r="C20" s="42"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="43"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -2006,7 +2016,7 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9"/>
       <c r="B21" s="8"/>
       <c r="C21" s="15"/>
@@ -2051,7 +2061,7 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="B22" s="8"/>
       <c r="C22" s="15"/>
@@ -2096,7 +2106,7 @@
       <c r="AP22"/>
       <c r="AQ22"/>
     </row>
-    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9"/>
       <c r="B23" s="8"/>
       <c r="C23" s="15"/>
@@ -2141,7 +2151,7 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9"/>
       <c r="B24" s="8"/>
       <c r="C24" s="15"/>
@@ -2186,7 +2196,7 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9"/>
       <c r="B25" s="8"/>
       <c r="C25" s="15"/>
@@ -2231,7 +2241,7 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9"/>
       <c r="B26" s="8"/>
       <c r="C26" s="15"/>
@@ -2276,7 +2286,7 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9"/>
       <c r="B27" s="8"/>
       <c r="C27" s="15"/>
@@ -2321,17 +2331,17 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="18">
-      <c r="A28" s="33" t="s">
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A28" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="B28" s="34"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="34"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="35"/>
+      <c r="B28" s="42"/>
+      <c r="C28" s="42"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="42"/>
+      <c r="G28" s="42"/>
+      <c r="H28" s="43"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2368,7 +2378,7 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9"/>
       <c r="B29" s="8"/>
       <c r="C29" s="15"/>
@@ -2413,7 +2423,7 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9"/>
       <c r="B30" s="8"/>
       <c r="C30" s="15"/>
@@ -2458,7 +2468,7 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9"/>
       <c r="B31" s="8"/>
       <c r="C31" s="15"/>
@@ -2505,7 +2515,7 @@
       <c r="AP31"/>
       <c r="AQ31"/>
     </row>
-    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
       <c r="B32" s="8"/>
       <c r="C32" s="15"/>
@@ -2550,7 +2560,7 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9"/>
       <c r="B33" s="8"/>
       <c r="C33" s="15"/>
@@ -2595,7 +2605,7 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="9"/>
       <c r="B34" s="8"/>
       <c r="C34" s="15"/>
@@ -2640,7 +2650,7 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1">
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="10"/>
       <c r="B35" s="11"/>
       <c r="C35" s="17"/>
@@ -2685,7 +2695,7 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" s="2" customFormat="1" ht="13.5">
+    <row r="36" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A36" s="5"/>
       <c r="B36" s="3"/>
       <c r="C36" s="4"/>
@@ -2730,59 +2740,54 @@
       <c r="AP36"/>
       <c r="AQ36"/>
     </row>
-    <row r="37" spans="1:43" customFormat="1"/>
-    <row r="38" spans="1:43" customFormat="1"/>
-    <row r="39" spans="1:43" customFormat="1"/>
-    <row r="40" spans="1:43" customFormat="1"/>
-    <row r="41" spans="1:43" customFormat="1"/>
-    <row r="42" spans="1:43" customFormat="1"/>
-    <row r="43" spans="1:43" customFormat="1"/>
-    <row r="44" spans="1:43" customFormat="1"/>
-    <row r="45" spans="1:43" customFormat="1"/>
-    <row r="46" spans="1:43" customFormat="1"/>
-    <row r="47" spans="1:43" customFormat="1"/>
-    <row r="48" spans="1:43" customFormat="1"/>
-    <row r="49" customFormat="1"/>
-    <row r="50" customFormat="1"/>
-    <row r="51" customFormat="1"/>
-    <row r="52" customFormat="1"/>
-    <row r="53" customFormat="1"/>
-    <row r="54" customFormat="1"/>
-    <row r="55" customFormat="1"/>
-    <row r="56" customFormat="1"/>
-    <row r="57" customFormat="1"/>
-    <row r="58" customFormat="1"/>
-    <row r="59" customFormat="1"/>
-    <row r="60" customFormat="1"/>
-    <row r="61" customFormat="1"/>
-    <row r="62" customFormat="1"/>
-    <row r="63" customFormat="1"/>
-    <row r="64" customFormat="1"/>
-    <row r="65" customFormat="1"/>
-    <row r="66" customFormat="1"/>
-    <row r="67" customFormat="1"/>
-    <row r="68" customFormat="1"/>
-    <row r="69" customFormat="1"/>
-    <row r="70" customFormat="1"/>
-    <row r="71" customFormat="1"/>
-    <row r="72" customFormat="1"/>
-    <row r="73" customFormat="1"/>
-    <row r="74" customFormat="1"/>
-    <row r="75" customFormat="1"/>
-    <row r="76" customFormat="1"/>
-    <row r="77" customFormat="1"/>
-    <row r="78" customFormat="1"/>
-    <row r="79" customFormat="1"/>
-    <row r="80" customFormat="1"/>
-    <row r="81" customFormat="1"/>
-    <row r="82" customFormat="1"/>
+    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="62" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="63" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="65" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="67" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="68" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="69" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="70" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="71" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="72" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="73" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="74" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="75" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="77" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="78" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="79" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2790,6 +2795,11 @@
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2800,6 +2810,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a81de258-2782-43d6-9d1d-cd28d60619af">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009F94F24C812C1443AF756F3262092C76" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="151ba19e32653bee0a5eee1707588175">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a81de258-2782-43d6-9d1d-cd28d60619af" xmlns:ns3="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="177f0ace5463b349477f87f1b4642be3" ns2:_="" ns3:_="">
     <xsd:import namespace="a81de258-2782-43d6-9d1d-cd28d60619af"/>
@@ -3000,17 +3021,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a81de258-2782-43d6-9d1d-cd28d60619af">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -3021,13 +3031,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E8AC1FA-2BD8-42E8-B266-319DE6BBF638}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76E9F743-2553-4538-B86E-9E9E949B7313}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a81de258-2782-43d6-9d1d-cd28d60619af"/>
+    <ds:schemaRef ds:uri="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76E9F743-2553-4538-B86E-9E9E949B7313}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E8AC1FA-2BD8-42E8-B266-319DE6BBF638}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="a81de258-2782-43d6-9d1d-cd28d60619af"/>
+    <ds:schemaRef ds:uri="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AE36CC0-C123-4309-B645-BEFA7CB5FE5A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AE36CC0-C123-4309-B645-BEFA7CB5FE5A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>